<commit_message>
decaf-tax post: refresh mascetti decaf_2025.{xlsx,pdf} dopo passaggio a LIFO
I due file nel bundle del blog erano stati generati prima della
conversione di forex_gains.py da FIFO unificato a LIFO per singolo
conto (commit decaf 9c07d14 e successivo regen examples e30b940).

Il PDF e l'Excel di mascetti 2025 nel bundle erano quindi stantii
rispetto agli output committati in examples/mascetti/ del repo decaf.
Li allineo copiando i freschi 2025.{xlsx,pdf} da
/home/vjt/code/decaf/examples/mascetti/.

Il YAML non e' servito nel bundle (si linka da GitHub), solo i due
file binari che il lettore puo' scaricare direttamente dalla pagina
del post.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/posts/2026-04-18-decaf-tax/decaf_2025.xlsx
+++ b/content/posts/2026-04-18-decaf-tax/decaf_2025.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>-99.34999999999999</v>
+        <v>488.64</v>
       </c>
     </row>
     <row r="15">
@@ -1842,18 +1842,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -2148,12 +2148,12 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
+          <t>Plusvalenza valutaria USD (LIFO per conto)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2025-04-03</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2162,16 +2162,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>13350</v>
+        <v>80000</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>11773.53</v>
+        <v>70552.96000000001</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>12388.64</v>
+        <v>72091.56</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>-615.12</v>
+        <v>-1538.6</v>
       </c>
       <c r="J6" t="n">
         <v>1.1339</v>
@@ -2197,33 +2197,33 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
+          <t>Plusvalenza valutaria USD (LIFO per conto)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2024-06-10</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-10-25</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>50</v>
+        <v>2400</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>44.1</v>
+        <v>2066.83</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>46.49</v>
+        <v>2065.05</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>-2.39</v>
+        <v>1.78</v>
       </c>
       <c r="J7" t="n">
-        <v>1.1339</v>
+        <v>1.1612</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -2238,366 +2238,23 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2024-06-24</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>2116.59</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>2236.72</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>-120.13</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1.1339</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="I8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2024-08-20</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>45</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>39.69</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>40.6</v>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NETTO</t>
+        </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>-0.91</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1.1339</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2024-09-10</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>1650</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>1455.15</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>1495.78</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>-40.63</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1.1339</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2024-11-15</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>40</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>35.28</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>-2.52</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1.1339</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2025-03-11</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>2645.74</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>2749.27</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>-103.53</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1.1339</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2025-04-03</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>59465</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>52442.9</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>53586.55</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>-1143.66</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1.1339</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>EUR.USD</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2025-04-03</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2025-10-25</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>2066.83</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>2162.75</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>-95.92</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1.1612</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="I15" s="6" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>NETTO</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>-99.34999999999999</v>
+        <v>488.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>